<commit_message>
Updates to switch between local and openai
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/satish_byndr/Documents/workspace-py/wot-poc/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82814484-919F-9F46-8E1C-22AAB28463FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="DID Data" sheetId="1" r:id="rId4"/>
+    <sheet name="DID Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -703,44 +712,69 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -748,72 +782,55 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1003,26 +1020,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:BY12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="39.88"/>
-    <col customWidth="1" min="5" max="5" width="19.25"/>
-    <col customWidth="1" min="6" max="6" width="18.75"/>
-    <col customWidth="1" min="7" max="7" width="19.13"/>
-    <col customWidth="1" min="8" max="8" width="16.13"/>
-    <col customWidth="1" min="30" max="30" width="22.38"/>
-    <col customWidth="1" min="31" max="31" width="18.5"/>
+    <col min="3" max="3" width="39.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.1640625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.1640625" customWidth="1"/>
+    <col min="8" max="8" width="16.1640625" customWidth="1"/>
+    <col min="30" max="30" width="22.33203125" customWidth="1"/>
+    <col min="31" max="31" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1249,12 +1269,12 @@
       <c r="BX1" s="1"/>
       <c r="BY1" s="1"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B2" s="2">
-        <v>275.0</v>
+        <v>275</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>74</v>
@@ -1272,7 +1292,7 @@
         <v>78</v>
       </c>
       <c r="H2" s="2">
-        <v>2022.0</v>
+        <v>2022</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>79</v>
@@ -1281,7 +1301,7 @@
         <v>80</v>
       </c>
       <c r="K2" s="2">
-        <v>2022.0</v>
+        <v>2022</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>79</v>
@@ -1316,7 +1336,7 @@
       <c r="V2" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="W2" s="4"/>
+      <c r="W2" s="2"/>
       <c r="X2" s="2" t="s">
         <v>84</v>
       </c>
@@ -1329,21 +1349,21 @@
       <c r="AA2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
       <c r="AD2" s="2" t="s">
         <v>91</v>
       </c>
       <c r="AE2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
+      <c r="AF2" s="2"/>
+      <c r="AG2" s="2"/>
       <c r="AH2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="4"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
       <c r="AK2" s="2" t="s">
         <v>84</v>
       </c>
@@ -1374,43 +1394,43 @@
       <c r="AT2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AU2" s="5" t="s">
+      <c r="AU2" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="AV2" s="6" t="s">
+      <c r="AV2" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="AW2" s="4"/>
-      <c r="AX2" s="4"/>
-      <c r="AY2" s="4"/>
+      <c r="AW2" s="2"/>
+      <c r="AX2" s="2"/>
+      <c r="AY2" s="2"/>
       <c r="AZ2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="BA2" s="6" t="s">
+      <c r="BA2" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="BB2" s="6" t="s">
+      <c r="BB2" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="BC2" s="4"/>
-      <c r="BD2" s="4"/>
-      <c r="BE2" s="4"/>
+      <c r="BC2" s="2"/>
+      <c r="BD2" s="2"/>
+      <c r="BE2" s="2"/>
       <c r="BF2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="BG2" s="6" t="s">
+      <c r="BG2" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="BH2" s="6" t="s">
+      <c r="BH2" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="BI2" s="7" t="s">
+      <c r="BI2" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="BJ2" s="6" t="s">
+      <c r="BJ2" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="BK2" s="6" t="s">
+      <c r="BK2" s="5" t="s">
         <v>88</v>
       </c>
       <c r="BL2" s="3" t="s">
@@ -1425,37 +1445,37 @@
       <c r="BO2" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="BP2" s="8" t="s">
+      <c r="BP2" s="2" t="s">
         <v>107</v>
       </c>
       <c r="BQ2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BR2" s="6" t="s">
+      <c r="BR2" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="BS2" s="6" t="s">
+      <c r="BS2" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="BT2" s="8" t="s">
+      <c r="BT2" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="BU2" s="9" t="s">
+      <c r="BU2" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="BV2" s="9" t="s">
+      <c r="BV2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="BW2" s="4"/>
-      <c r="BX2" s="4"/>
-      <c r="BY2" s="4"/>
+      <c r="BW2" s="2"/>
+      <c r="BX2" s="2"/>
+      <c r="BY2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>113</v>
       </c>
       <c r="B3" s="2">
-        <v>281.0</v>
+        <v>281</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>114</v>
@@ -1473,7 +1493,7 @@
         <v>118</v>
       </c>
       <c r="H3" s="2">
-        <v>2019.0</v>
+        <v>2019</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>117</v>
@@ -1482,7 +1502,7 @@
         <v>118</v>
       </c>
       <c r="K3" s="2">
-        <v>2019.0</v>
+        <v>2019</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>117</v>
@@ -1544,13 +1564,13 @@
       <c r="AE3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AF3" s="4"/>
-      <c r="AG3" s="4"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
       <c r="AH3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AI3" s="4"/>
-      <c r="AJ3" s="4"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
       <c r="AK3" s="2" t="s">
         <v>84</v>
       </c>
@@ -1581,82 +1601,82 @@
       <c r="AT3" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AU3" s="6" t="s">
+      <c r="AU3" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="AV3" s="6" t="s">
+      <c r="AV3" s="5" t="s">
         <v>131</v>
       </c>
       <c r="AW3" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AX3" s="4"/>
+      <c r="AX3" s="2"/>
       <c r="AY3" s="3" t="s">
         <v>133</v>
       </c>
       <c r="AZ3" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="BA3" s="6" t="s">
+      <c r="BA3" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="BB3" s="6" t="s">
+      <c r="BB3" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="BC3" s="4"/>
-      <c r="BD3" s="4"/>
-      <c r="BE3" s="4"/>
-      <c r="BF3" s="4"/>
-      <c r="BG3" s="4"/>
-      <c r="BH3" s="4"/>
-      <c r="BI3" s="4"/>
-      <c r="BJ3" s="4"/>
-      <c r="BK3" s="4"/>
+      <c r="BC3" s="2"/>
+      <c r="BD3" s="2"/>
+      <c r="BE3" s="2"/>
+      <c r="BF3" s="2"/>
+      <c r="BG3" s="2"/>
+      <c r="BH3" s="2"/>
+      <c r="BI3" s="2"/>
+      <c r="BJ3" s="2"/>
+      <c r="BK3" s="2"/>
       <c r="BL3" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="BM3" s="10" t="s">
+      <c r="BM3" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="BN3" s="6" t="s">
+      <c r="BN3" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="BO3" s="6" t="s">
+      <c r="BO3" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="BP3" s="8" t="s">
+      <c r="BP3" s="2" t="s">
         <v>140</v>
       </c>
       <c r="BQ3" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="BR3" s="6" t="s">
+      <c r="BR3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="BS3" s="6" t="s">
+      <c r="BS3" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="BT3" s="8" t="s">
+      <c r="BT3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="BU3" s="9" t="s">
+      <c r="BU3" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="BV3" s="9" t="s">
+      <c r="BV3" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="BW3" s="4"/>
-      <c r="BX3" s="4"/>
-      <c r="BY3" s="4"/>
+      <c r="BW3" s="2"/>
+      <c r="BX3" s="2"/>
+      <c r="BY3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>145</v>
       </c>
       <c r="B4" s="2">
-        <v>319.0</v>
-      </c>
-      <c r="C4" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>146</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -1665,14 +1685,14 @@
       <c r="E4" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="9" t="s">
         <v>149</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>150</v>
       </c>
       <c r="H4" s="2">
-        <v>2020.0</v>
+        <v>2020</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>151</v>
@@ -1681,7 +1701,7 @@
         <v>152</v>
       </c>
       <c r="K4" s="2">
-        <v>2020.0</v>
+        <v>2020</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>153</v>
@@ -1722,7 +1742,7 @@
       <c r="X4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="Y4" s="3" t="s">
+      <c r="Y4" s="9" t="s">
         <v>162</v>
       </c>
       <c r="Z4" s="3" t="s">
@@ -1731,7 +1751,7 @@
       <c r="AA4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AB4" s="4"/>
+      <c r="AB4" s="2"/>
       <c r="AC4" s="3" t="s">
         <v>164</v>
       </c>
@@ -1741,7 +1761,7 @@
       <c r="AE4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AF4" s="4"/>
+      <c r="AF4" s="2"/>
       <c r="AG4" s="3" t="s">
         <v>165</v>
       </c>
@@ -1757,112 +1777,112 @@
       <c r="AK4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AL4" s="4"/>
+      <c r="AL4" s="2"/>
       <c r="AM4" s="3" t="s">
         <v>167</v>
       </c>
       <c r="AN4" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AO4" s="4"/>
+      <c r="AO4" s="2"/>
       <c r="AP4" s="3" t="s">
         <v>164</v>
       </c>
       <c r="AQ4" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AR4" s="4"/>
+      <c r="AR4" s="2"/>
       <c r="AS4" s="3" t="s">
         <v>164</v>
       </c>
       <c r="AT4" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="AU4" s="6" t="s">
+      <c r="AU4" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="AV4" s="6" t="s">
+      <c r="AV4" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="AW4" s="4"/>
-      <c r="AX4" s="4"/>
-      <c r="AY4" s="4"/>
+      <c r="AW4" s="2"/>
+      <c r="AX4" s="2"/>
+      <c r="AY4" s="2"/>
       <c r="AZ4" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="BA4" s="6" t="s">
+      <c r="BA4" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="BB4" s="6" t="s">
+      <c r="BB4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="BC4" s="4"/>
-      <c r="BD4" s="4"/>
-      <c r="BE4" s="4"/>
+      <c r="BC4" s="2"/>
+      <c r="BD4" s="2"/>
+      <c r="BE4" s="2"/>
       <c r="BF4" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="BG4" s="6" t="s">
+      <c r="BG4" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="BH4" s="6" t="s">
+      <c r="BH4" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="BI4" s="7" t="s">
+      <c r="BI4" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="BJ4" s="6" t="s">
+      <c r="BJ4" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="BK4" s="4"/>
+      <c r="BK4" s="2"/>
       <c r="BL4" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="BM4" s="10" t="s">
+      <c r="BM4" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="BN4" s="6" t="s">
+      <c r="BN4" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="BO4" s="6" t="s">
+      <c r="BO4" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="BP4" s="8" t="s">
+      <c r="BP4" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="BQ4" s="8" t="s">
+      <c r="BQ4" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="BR4" s="6" t="s">
+      <c r="BR4" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="BS4" s="6" t="s">
+      <c r="BS4" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="BT4" s="8" t="s">
+      <c r="BT4" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="BU4" s="11" t="s">
+      <c r="BU4" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="BV4" s="11" t="s">
+      <c r="BV4" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="BW4" s="4"/>
-      <c r="BX4" s="4"/>
-      <c r="BY4" s="4"/>
+      <c r="BW4" s="2"/>
+      <c r="BX4" s="2"/>
+      <c r="BY4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>183</v>
       </c>
       <c r="B5" s="2">
-        <v>403.0</v>
+        <v>403</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D5" s="4"/>
+      <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
         <v>185</v>
       </c>
@@ -1873,7 +1893,7 @@
         <v>187</v>
       </c>
       <c r="H5" s="2">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>188</v>
@@ -1882,7 +1902,7 @@
         <v>189</v>
       </c>
       <c r="K5" s="2">
-        <v>2021.0</v>
+        <v>2021</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>186</v>
@@ -1953,7 +1973,7 @@
       <c r="AH5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AJ5" s="4"/>
+      <c r="AJ5" s="2"/>
       <c r="AK5" s="2" t="s">
         <v>93</v>
       </c>
@@ -1981,34 +2001,34 @@
       <c r="AS5" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="AT5" s="4"/>
-      <c r="AU5" s="4"/>
-      <c r="AV5" s="4"/>
-      <c r="AW5" s="4"/>
-      <c r="AX5" s="4"/>
-      <c r="AY5" s="4"/>
+      <c r="AT5" s="2"/>
+      <c r="AU5" s="2"/>
+      <c r="AV5" s="2"/>
+      <c r="AW5" s="2"/>
+      <c r="AX5" s="2"/>
+      <c r="AY5" s="2"/>
       <c r="AZ5" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="BA5" s="11" t="s">
+      <c r="BA5" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="BB5" s="11" t="s">
+      <c r="BB5" s="8" t="s">
         <v>208</v>
       </c>
       <c r="BC5" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="BD5" s="11" t="s">
+      <c r="BD5" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="BE5" s="11" t="s">
+      <c r="BE5" s="8" t="s">
         <v>211</v>
       </c>
       <c r="BF5" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="BG5" s="11" t="s">
+      <c r="BG5" s="8" t="s">
         <v>212</v>
       </c>
       <c r="BH5" s="3" t="s">
@@ -2017,10 +2037,10 @@
       <c r="BI5" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="BJ5" s="11" t="s">
+      <c r="BJ5" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="BK5" s="11" t="s">
+      <c r="BK5" s="8" t="s">
         <v>215</v>
       </c>
       <c r="BL5" s="3" t="s">
@@ -2029,10 +2049,10 @@
       <c r="BM5" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="BN5" s="11" t="s">
+      <c r="BN5" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="BO5" s="11" t="s">
+      <c r="BO5" s="8" t="s">
         <v>218</v>
       </c>
       <c r="BP5" s="2" t="s">
@@ -2047,422 +2067,422 @@
       <c r="BS5" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="BT5" s="8" t="s">
+      <c r="BT5" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="BU5" s="9" t="s">
+      <c r="BU5" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="BV5" s="9" t="s">
+      <c r="BV5" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="BW5" s="4"/>
-      <c r="BX5" s="4"/>
-      <c r="BY5" s="4"/>
+      <c r="BW5" s="2"/>
+      <c r="BX5" s="2"/>
+      <c r="BY5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
-      <c r="Z6" s="4"/>
-      <c r="AA6" s="4"/>
-      <c r="AB6" s="4"/>
-      <c r="AC6" s="4"/>
-      <c r="AD6" s="4"/>
-      <c r="AE6" s="4"/>
-      <c r="AF6" s="4"/>
-      <c r="AG6" s="4"/>
-      <c r="AH6" s="4"/>
-      <c r="AI6" s="4"/>
-      <c r="AJ6" s="4"/>
-      <c r="AK6" s="4"/>
-      <c r="AL6" s="4"/>
-      <c r="AM6" s="4"/>
-      <c r="AN6" s="4"/>
-      <c r="AO6" s="4"/>
-      <c r="AP6" s="4"/>
-      <c r="AQ6" s="4"/>
-      <c r="AR6" s="4"/>
-      <c r="AS6" s="4"/>
-      <c r="AT6" s="4"/>
-      <c r="AU6" s="4"/>
-      <c r="AV6" s="4"/>
-      <c r="AW6" s="4"/>
-      <c r="AX6" s="4"/>
-      <c r="AY6" s="4"/>
-      <c r="AZ6" s="4"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+      <c r="AK6" s="2"/>
+      <c r="AL6" s="2"/>
+      <c r="AM6" s="2"/>
+      <c r="AN6" s="2"/>
+      <c r="AO6" s="2"/>
+      <c r="AP6" s="2"/>
+      <c r="AQ6" s="2"/>
+      <c r="AR6" s="2"/>
+      <c r="AS6" s="2"/>
+      <c r="AT6" s="2"/>
+      <c r="AU6" s="2"/>
+      <c r="AV6" s="2"/>
+      <c r="AW6" s="2"/>
+      <c r="AX6" s="2"/>
+      <c r="AY6" s="2"/>
+      <c r="AZ6" s="2"/>
       <c r="BA6" s="2"/>
-      <c r="BC6" s="4"/>
-      <c r="BD6" s="4"/>
-      <c r="BE6" s="4"/>
+      <c r="BC6" s="2"/>
+      <c r="BD6" s="2"/>
+      <c r="BE6" s="2"/>
       <c r="BI6" s="2"/>
-      <c r="BJ6" s="4"/>
-      <c r="BK6" s="4"/>
-      <c r="BL6" s="4"/>
-      <c r="BM6" s="4"/>
-      <c r="BN6" s="4"/>
-      <c r="BO6" s="4"/>
-      <c r="BP6" s="4"/>
-      <c r="BQ6" s="4"/>
-      <c r="BR6" s="12"/>
-      <c r="BS6" s="12"/>
-      <c r="BT6" s="4"/>
-      <c r="BU6" s="4"/>
-      <c r="BV6" s="4"/>
-      <c r="BW6" s="4"/>
-      <c r="BX6" s="4"/>
-      <c r="BY6" s="4"/>
+      <c r="BJ6" s="2"/>
+      <c r="BK6" s="2"/>
+      <c r="BL6" s="2"/>
+      <c r="BM6" s="2"/>
+      <c r="BN6" s="2"/>
+      <c r="BO6" s="2"/>
+      <c r="BP6" s="2"/>
+      <c r="BQ6" s="2"/>
+      <c r="BR6" s="2"/>
+      <c r="BS6" s="2"/>
+      <c r="BT6" s="2"/>
+      <c r="BU6" s="2"/>
+      <c r="BV6" s="2"/>
+      <c r="BW6" s="2"/>
+      <c r="BX6" s="2"/>
+      <c r="BY6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
-      <c r="AA7" s="4"/>
-      <c r="AB7" s="4"/>
-      <c r="AC7" s="4"/>
-      <c r="AD7" s="4"/>
-      <c r="AE7" s="4"/>
-      <c r="AF7" s="4"/>
-      <c r="AG7" s="4"/>
-      <c r="AH7" s="4"/>
-      <c r="AI7" s="4"/>
-      <c r="AJ7" s="4"/>
-      <c r="AK7" s="4"/>
-      <c r="AL7" s="4"/>
-      <c r="AM7" s="4"/>
-      <c r="AN7" s="4"/>
-      <c r="AO7" s="4"/>
-      <c r="AP7" s="4"/>
-      <c r="AQ7" s="4"/>
-      <c r="AR7" s="4"/>
-      <c r="AS7" s="4"/>
-      <c r="AT7" s="4"/>
-      <c r="AU7" s="4"/>
-      <c r="AV7" s="4"/>
-      <c r="AW7" s="4"/>
-      <c r="AX7" s="4"/>
-      <c r="AY7" s="4"/>
-      <c r="AZ7" s="4"/>
-      <c r="BA7" s="4"/>
-      <c r="BB7" s="4"/>
-      <c r="BC7" s="4"/>
-      <c r="BD7" s="4"/>
-      <c r="BE7" s="4"/>
-      <c r="BF7" s="4"/>
-      <c r="BG7" s="4"/>
-      <c r="BH7" s="4"/>
-      <c r="BI7" s="4"/>
-      <c r="BJ7" s="4"/>
-      <c r="BK7" s="4"/>
-      <c r="BL7" s="4"/>
-      <c r="BM7" s="4"/>
-      <c r="BN7" s="4"/>
-      <c r="BO7" s="4"/>
-      <c r="BP7" s="4"/>
-      <c r="BQ7" s="4"/>
-      <c r="BR7" s="4"/>
-      <c r="BS7" s="4"/>
-      <c r="BT7" s="4"/>
-      <c r="BU7" s="4"/>
-      <c r="BV7" s="4"/>
-      <c r="BW7" s="4"/>
-      <c r="BX7" s="4"/>
-      <c r="BY7" s="4"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
+      <c r="AK7" s="2"/>
+      <c r="AL7" s="2"/>
+      <c r="AM7" s="2"/>
+      <c r="AN7" s="2"/>
+      <c r="AO7" s="2"/>
+      <c r="AP7" s="2"/>
+      <c r="AQ7" s="2"/>
+      <c r="AR7" s="2"/>
+      <c r="AS7" s="2"/>
+      <c r="AT7" s="2"/>
+      <c r="AU7" s="2"/>
+      <c r="AV7" s="2"/>
+      <c r="AW7" s="2"/>
+      <c r="AX7" s="2"/>
+      <c r="AY7" s="2"/>
+      <c r="AZ7" s="2"/>
+      <c r="BA7" s="2"/>
+      <c r="BB7" s="2"/>
+      <c r="BC7" s="2"/>
+      <c r="BD7" s="2"/>
+      <c r="BE7" s="2"/>
+      <c r="BF7" s="2"/>
+      <c r="BG7" s="2"/>
+      <c r="BH7" s="2"/>
+      <c r="BI7" s="2"/>
+      <c r="BJ7" s="2"/>
+      <c r="BK7" s="2"/>
+      <c r="BL7" s="2"/>
+      <c r="BM7" s="2"/>
+      <c r="BN7" s="2"/>
+      <c r="BO7" s="2"/>
+      <c r="BP7" s="2"/>
+      <c r="BQ7" s="2"/>
+      <c r="BR7" s="2"/>
+      <c r="BS7" s="2"/>
+      <c r="BT7" s="2"/>
+      <c r="BU7" s="2"/>
+      <c r="BV7" s="2"/>
+      <c r="BW7" s="2"/>
+      <c r="BX7" s="2"/>
+      <c r="BY7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
-      <c r="V8" s="4"/>
-      <c r="W8" s="4"/>
-      <c r="X8" s="4"/>
-      <c r="Y8" s="4"/>
-      <c r="Z8" s="4"/>
-      <c r="AA8" s="4"/>
-      <c r="AB8" s="4"/>
-      <c r="AC8" s="4"/>
-      <c r="AD8" s="4"/>
-      <c r="AE8" s="4"/>
-      <c r="AF8" s="4"/>
-      <c r="AG8" s="4"/>
-      <c r="AH8" s="4"/>
-      <c r="AI8" s="4"/>
-      <c r="AJ8" s="4"/>
-      <c r="AK8" s="4"/>
-      <c r="AL8" s="4"/>
-      <c r="AM8" s="4"/>
-      <c r="AN8" s="4"/>
-      <c r="AO8" s="4"/>
-      <c r="AP8" s="4"/>
-      <c r="AQ8" s="4"/>
-      <c r="AR8" s="4"/>
-      <c r="AS8" s="4"/>
-      <c r="AT8" s="4"/>
-      <c r="AU8" s="4"/>
-      <c r="AV8" s="4"/>
-      <c r="AW8" s="4"/>
-      <c r="AX8" s="4"/>
-      <c r="AY8" s="4"/>
-      <c r="AZ8" s="4"/>
-      <c r="BA8" s="4"/>
-      <c r="BB8" s="4"/>
-      <c r="BC8" s="4"/>
-      <c r="BD8" s="4"/>
-      <c r="BE8" s="4"/>
-      <c r="BF8" s="4"/>
-      <c r="BG8" s="4"/>
-      <c r="BH8" s="4"/>
-      <c r="BI8" s="4"/>
-      <c r="BJ8" s="4"/>
-      <c r="BK8" s="4"/>
-      <c r="BL8" s="4"/>
-      <c r="BM8" s="4"/>
-      <c r="BN8" s="4"/>
-      <c r="BO8" s="4"/>
-      <c r="BP8" s="4"/>
-      <c r="BQ8" s="4"/>
-      <c r="BR8" s="4"/>
-      <c r="BS8" s="4"/>
-      <c r="BT8" s="4"/>
-      <c r="BU8" s="4"/>
-      <c r="BV8" s="4"/>
-      <c r="BW8" s="4"/>
-      <c r="BX8" s="4"/>
-      <c r="BY8" s="4"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
+      <c r="AJ8" s="2"/>
+      <c r="AK8" s="2"/>
+      <c r="AL8" s="2"/>
+      <c r="AM8" s="2"/>
+      <c r="AN8" s="2"/>
+      <c r="AO8" s="2"/>
+      <c r="AP8" s="2"/>
+      <c r="AQ8" s="2"/>
+      <c r="AR8" s="2"/>
+      <c r="AS8" s="2"/>
+      <c r="AT8" s="2"/>
+      <c r="AU8" s="2"/>
+      <c r="AV8" s="2"/>
+      <c r="AW8" s="2"/>
+      <c r="AX8" s="2"/>
+      <c r="AY8" s="2"/>
+      <c r="AZ8" s="2"/>
+      <c r="BA8" s="2"/>
+      <c r="BB8" s="2"/>
+      <c r="BC8" s="2"/>
+      <c r="BD8" s="2"/>
+      <c r="BE8" s="2"/>
+      <c r="BF8" s="2"/>
+      <c r="BG8" s="2"/>
+      <c r="BH8" s="2"/>
+      <c r="BI8" s="2"/>
+      <c r="BJ8" s="2"/>
+      <c r="BK8" s="2"/>
+      <c r="BL8" s="2"/>
+      <c r="BM8" s="2"/>
+      <c r="BN8" s="2"/>
+      <c r="BO8" s="2"/>
+      <c r="BP8" s="2"/>
+      <c r="BQ8" s="2"/>
+      <c r="BR8" s="2"/>
+      <c r="BS8" s="2"/>
+      <c r="BT8" s="2"/>
+      <c r="BU8" s="2"/>
+      <c r="BV8" s="2"/>
+      <c r="BW8" s="2"/>
+      <c r="BX8" s="2"/>
+      <c r="BY8" s="2"/>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="12">
-      <c r="BU12" s="13"/>
+    <row r="12" spans="1:77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="BU12" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C2"/>
-    <hyperlink r:id="rId2" ref="D2"/>
-    <hyperlink r:id="rId3" ref="F2"/>
-    <hyperlink r:id="rId4" location="selection-579.62-579.204" ref="G2"/>
-    <hyperlink r:id="rId5" ref="I2"/>
-    <hyperlink r:id="rId6" location="selection-2077.79-2077.338" ref="J2"/>
-    <hyperlink r:id="rId7" ref="L2"/>
-    <hyperlink r:id="rId8" location="selection-2077.79-2077.338" ref="M2"/>
-    <hyperlink r:id="rId9" ref="O2"/>
-    <hyperlink r:id="rId10" ref="P2"/>
-    <hyperlink r:id="rId11" ref="R2"/>
-    <hyperlink r:id="rId12" location="selection-2831.0-2842.0" ref="S2"/>
-    <hyperlink r:id="rId13" ref="U2"/>
-    <hyperlink r:id="rId14" location="selection-657.0-671.225" ref="V2"/>
-    <hyperlink r:id="rId15" ref="Y2"/>
-    <hyperlink r:id="rId16" location="selection-949.0-949.92" ref="Z2"/>
-    <hyperlink r:id="rId17" ref="AL2"/>
-    <hyperlink r:id="rId18" location="selection-643.0-657.225" ref="AM2"/>
-    <hyperlink r:id="rId19" ref="AO2"/>
-    <hyperlink r:id="rId20" location="selection-505.0-509.414" ref="AP2"/>
-    <hyperlink r:id="rId21" ref="AR2"/>
-    <hyperlink r:id="rId22" location="selection-505.0-509.414" ref="AS2"/>
-    <hyperlink r:id="rId23" location="selection-2555.0-2846.1" ref="AU2"/>
-    <hyperlink r:id="rId24" ref="AV2"/>
-    <hyperlink r:id="rId25" location="selection-2555.0-2846.1" ref="BA2"/>
-    <hyperlink r:id="rId26" ref="BB2"/>
-    <hyperlink r:id="rId27" ref="BG2"/>
-    <hyperlink r:id="rId28" location="selection-921.129-921.457" ref="BH2"/>
-    <hyperlink r:id="rId29" location="selection-1003.0-1003.32" ref="BJ2"/>
-    <hyperlink r:id="rId30" ref="BK2"/>
-    <hyperlink r:id="rId31" ref="BL2"/>
-    <hyperlink r:id="rId32" location="selection-941.0-941.46" ref="BN2"/>
-    <hyperlink r:id="rId33" ref="BO2"/>
-    <hyperlink r:id="rId34" location="selection-2127.0-2132.0" ref="BR2"/>
-    <hyperlink r:id="rId35" ref="BS2"/>
-    <hyperlink r:id="rId36" location="selection-2131.0-2131.717" ref="BU2"/>
-    <hyperlink r:id="rId37" ref="BV2"/>
-    <hyperlink r:id="rId38" ref="C3"/>
-    <hyperlink r:id="rId39" ref="D3"/>
-    <hyperlink r:id="rId40" ref="F3"/>
-    <hyperlink r:id="rId41" ref="G3"/>
-    <hyperlink r:id="rId42" ref="I3"/>
-    <hyperlink r:id="rId43" ref="J3"/>
-    <hyperlink r:id="rId44" ref="L3"/>
-    <hyperlink r:id="rId45" ref="M3"/>
-    <hyperlink r:id="rId46" ref="O3"/>
-    <hyperlink r:id="rId47" ref="P3"/>
-    <hyperlink r:id="rId48" ref="R3"/>
-    <hyperlink r:id="rId49" location="selection-1013.0-1013.80" ref="S3"/>
-    <hyperlink r:id="rId50" ref="U3"/>
-    <hyperlink r:id="rId51" location="selection-2307.0-2327.221" ref="V3"/>
-    <hyperlink r:id="rId52" ref="W3"/>
-    <hyperlink r:id="rId53" ref="Y3"/>
-    <hyperlink r:id="rId54" location="69%" ref="Z3"/>
-    <hyperlink r:id="rId55" ref="AB3"/>
-    <hyperlink r:id="rId56" location="selection-2307.0-2327.221" ref="AC3"/>
-    <hyperlink r:id="rId57" ref="AL3"/>
-    <hyperlink r:id="rId58" location="selection-463.0-493.112" ref="AM3"/>
-    <hyperlink r:id="rId59" ref="AO3"/>
-    <hyperlink r:id="rId60" location="selection-2359.0-2365.220" ref="AP3"/>
-    <hyperlink r:id="rId61" ref="AR3"/>
-    <hyperlink r:id="rId62" location="selection-2359.0-2365.220" ref="AS3"/>
-    <hyperlink r:id="rId63" location="selection-323.0-323.57" ref="AU3"/>
-    <hyperlink r:id="rId64" ref="AV3"/>
-    <hyperlink r:id="rId65" ref="AY3"/>
-    <hyperlink r:id="rId66" ref="BA3"/>
-    <hyperlink r:id="rId67" ref="BB3"/>
-    <hyperlink r:id="rId68" ref="BL3"/>
-    <hyperlink r:id="rId69" location="selection-2359.0-2359.517" ref="BN3"/>
-    <hyperlink r:id="rId70" ref="BO3"/>
-    <hyperlink r:id="rId71" location="selection-517.0-527.14" ref="BR3"/>
-    <hyperlink r:id="rId72" ref="BS3"/>
-    <hyperlink r:id="rId73" ref="BU3"/>
-    <hyperlink r:id="rId74" ref="BV3"/>
-    <hyperlink r:id="rId75" ref="C4"/>
-    <hyperlink r:id="rId76" ref="D4"/>
-    <hyperlink r:id="rId77" ref="F4"/>
-    <hyperlink r:id="rId78" ref="G4"/>
-    <hyperlink r:id="rId79" ref="I4"/>
-    <hyperlink r:id="rId80" ref="J4"/>
-    <hyperlink r:id="rId81" ref="L4"/>
-    <hyperlink r:id="rId82" ref="M4"/>
-    <hyperlink r:id="rId83" ref="O4"/>
-    <hyperlink r:id="rId84" ref="P4"/>
-    <hyperlink r:id="rId85" ref="R4"/>
-    <hyperlink r:id="rId86" location="selection-1081.45-1081.52" ref="S4"/>
-    <hyperlink r:id="rId87" ref="U4"/>
-    <hyperlink r:id="rId88" ref="V4"/>
-    <hyperlink r:id="rId89" ref="W4"/>
-    <hyperlink r:id="rId90" ref="Y4"/>
-    <hyperlink r:id="rId91" ref="Z4"/>
-    <hyperlink r:id="rId92" ref="AC4"/>
-    <hyperlink r:id="rId93" ref="AG4"/>
-    <hyperlink r:id="rId94" ref="AI4"/>
-    <hyperlink r:id="rId95" location="selection-2343.81-2437.13" ref="AJ4"/>
-    <hyperlink r:id="rId96" ref="AM4"/>
-    <hyperlink r:id="rId97" ref="AP4"/>
-    <hyperlink r:id="rId98" ref="AS4"/>
-    <hyperlink r:id="rId99" ref="AU4"/>
-    <hyperlink r:id="rId100" ref="AV4"/>
-    <hyperlink r:id="rId101" location="selection-1653.0-1657.338" ref="BA4"/>
-    <hyperlink r:id="rId102" ref="BB4"/>
-    <hyperlink r:id="rId103" ref="BG4"/>
-    <hyperlink r:id="rId104" ref="BH4"/>
-    <hyperlink r:id="rId105" ref="BJ4"/>
-    <hyperlink r:id="rId106" ref="BL4"/>
-    <hyperlink r:id="rId107" location="selection-1997.409-1997.473" ref="BN4"/>
-    <hyperlink r:id="rId108" ref="BO4"/>
-    <hyperlink r:id="rId109" location="selection-755.0-864.1" ref="BR4"/>
-    <hyperlink r:id="rId110" ref="BS4"/>
-    <hyperlink r:id="rId111" ref="BU4"/>
-    <hyperlink r:id="rId112" ref="BV4"/>
-    <hyperlink r:id="rId113" ref="C5"/>
-    <hyperlink r:id="rId114" ref="F5"/>
-    <hyperlink r:id="rId115" ref="G5"/>
-    <hyperlink r:id="rId116" ref="I5"/>
-    <hyperlink r:id="rId117" ref="J5"/>
-    <hyperlink r:id="rId118" ref="L5"/>
-    <hyperlink r:id="rId119" ref="M5"/>
-    <hyperlink r:id="rId120" ref="O5"/>
-    <hyperlink r:id="rId121" ref="P5"/>
-    <hyperlink r:id="rId122" ref="R5"/>
-    <hyperlink r:id="rId123" ref="S5"/>
-    <hyperlink r:id="rId124" ref="U5"/>
-    <hyperlink r:id="rId125" ref="V5"/>
-    <hyperlink r:id="rId126" ref="W5"/>
-    <hyperlink r:id="rId127" ref="Y5"/>
-    <hyperlink r:id="rId128" ref="Z5"/>
-    <hyperlink r:id="rId129" ref="AB5"/>
-    <hyperlink r:id="rId130" ref="AC5"/>
-    <hyperlink r:id="rId131" ref="AF5"/>
-    <hyperlink r:id="rId132" ref="AG5"/>
-    <hyperlink r:id="rId133" ref="AL5"/>
-    <hyperlink r:id="rId134" ref="AM5"/>
-    <hyperlink r:id="rId135" ref="AO5"/>
-    <hyperlink r:id="rId136" ref="AP5"/>
-    <hyperlink r:id="rId137" ref="AR5"/>
-    <hyperlink r:id="rId138" ref="AS5"/>
-    <hyperlink r:id="rId139" ref="BA5"/>
-    <hyperlink r:id="rId140" ref="BB5"/>
-    <hyperlink r:id="rId141" location="ecosystem" ref="BD5"/>
-    <hyperlink r:id="rId142" ref="BE5"/>
-    <hyperlink r:id="rId143" location="selection-2287.0-2287.36" ref="BG5"/>
-    <hyperlink r:id="rId144" ref="BH5"/>
-    <hyperlink r:id="rId145" ref="BJ5"/>
-    <hyperlink r:id="rId146" location="rationale-for-using-the-cosmos-blockchain-framework-for-cheqd" ref="BK5"/>
-    <hyperlink r:id="rId147" ref="BL5"/>
-    <hyperlink r:id="rId148" location="selection-2519.0-2519.186" ref="BN5"/>
-    <hyperlink r:id="rId149" ref="BO5"/>
-    <hyperlink r:id="rId150" ref="BR5"/>
-    <hyperlink r:id="rId151" ref="BS5"/>
-    <hyperlink r:id="rId152" ref="BU5"/>
-    <hyperlink r:id="rId153" ref="BV5"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F2" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G2" r:id="rId4" location="selection-579.62-579.204" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="I2" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J2" r:id="rId6" location="selection-2077.79-2077.338" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="L2" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="M2" r:id="rId8" location="selection-2077.79-2077.338" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="O2" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="P2" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="R2" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="S2" r:id="rId12" location="selection-2831.0-2842.0" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="U2" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="V2" r:id="rId14" location="selection-657.0-671.225" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="Y2" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="Z2" r:id="rId16" location="selection-949.0-949.92" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="AL2" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="AM2" r:id="rId18" location="selection-643.0-657.225" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="AO2" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="AP2" r:id="rId20" location="selection-505.0-509.414" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="AR2" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="AS2" r:id="rId22" location="selection-505.0-509.414" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="AU2" r:id="rId23" location="selection-2555.0-2846.1" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="AV2" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="BA2" r:id="rId25" location="selection-2555.0-2846.1" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="BB2" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="BG2" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="BH2" r:id="rId28" location="selection-921.129-921.457" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="BJ2" r:id="rId29" location="selection-1003.0-1003.32" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="BK2" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="BL2" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="BN2" r:id="rId32" location="selection-941.0-941.46" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="BO2" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="BR2" r:id="rId34" location="selection-2127.0-2132.0" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="BS2" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="BU2" r:id="rId36" location="selection-2131.0-2131.717" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="BV2" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="C3" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="D3" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="F3" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="G3" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="I3" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="J3" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="L3" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="M3" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="O3" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="P3" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="R3" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="S3" r:id="rId49" location="selection-1013.0-1013.80" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="U3" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="V3" r:id="rId51" location="selection-2307.0-2327.221" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="W3" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="Y3" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="Z3" r:id="rId54" location="69%" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="AB3" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="AC3" r:id="rId56" location="selection-2307.0-2327.221" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="AL3" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="AM3" r:id="rId58" location="selection-463.0-493.112" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="AO3" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="AP3" r:id="rId60" location="selection-2359.0-2365.220" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="AR3" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="AS3" r:id="rId62" location="selection-2359.0-2365.220" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="AU3" r:id="rId63" location="selection-323.0-323.57" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="AV3" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="AY3" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="BA3" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="BB3" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="BL3" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="BN3" r:id="rId69" location="selection-2359.0-2359.517" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="BO3" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="BR3" r:id="rId71" location="selection-517.0-527.14" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="BS3" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="BU3" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="BV3" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="C4" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="D4" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="F4" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="G4" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="I4" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="J4" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="L4" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="M4" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="O4" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="P4" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="R4" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="S4" r:id="rId86" location="selection-1081.45-1081.52" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="U4" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="V4" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="W4" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="Y4" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="Z4" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="AC4" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="AG4" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="AI4" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="AJ4" r:id="rId95" location="selection-2343.81-2437.13" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="AM4" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="AP4" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="AS4" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="AU4" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="AV4" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="BA4" r:id="rId101" location="selection-1653.0-1657.338" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="BB4" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="BG4" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="BH4" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="BJ4" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="BL4" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="BN4" r:id="rId107" location="selection-1997.409-1997.473" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="BO4" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="BR4" r:id="rId109" location="selection-755.0-864.1" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="BS4" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="BU4" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="BV4" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="C5" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="F5" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="G5" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="I5" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="J5" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="L5" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="M5" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="O5" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="P5" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="R5" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="S5" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="U5" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="V5" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="W5" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="Y5" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="Z5" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="AB5" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="AC5" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="AF5" r:id="rId131" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
+    <hyperlink ref="AG5" r:id="rId132" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
+    <hyperlink ref="AL5" r:id="rId133" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
+    <hyperlink ref="AM5" r:id="rId134" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
+    <hyperlink ref="AO5" r:id="rId135" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
+    <hyperlink ref="AP5" r:id="rId136" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
+    <hyperlink ref="AR5" r:id="rId137" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
+    <hyperlink ref="AS5" r:id="rId138" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
+    <hyperlink ref="BA5" r:id="rId139" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
+    <hyperlink ref="BB5" r:id="rId140" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
+    <hyperlink ref="BD5" r:id="rId141" location="ecosystem" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
+    <hyperlink ref="BE5" r:id="rId142" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
+    <hyperlink ref="BG5" r:id="rId143" location="selection-2287.0-2287.36" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
+    <hyperlink ref="BH5" r:id="rId144" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
+    <hyperlink ref="BJ5" r:id="rId145" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
+    <hyperlink ref="BK5" r:id="rId146" location="rationale-for-using-the-cosmos-blockchain-framework-for-cheqd" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
+    <hyperlink ref="BL5" r:id="rId147" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
+    <hyperlink ref="BN5" r:id="rId148" location="selection-2519.0-2519.186" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
+    <hyperlink ref="BO5" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
+    <hyperlink ref="BR5" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
+    <hyperlink ref="BS5" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
+    <hyperlink ref="BU5" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
+    <hyperlink ref="BV5" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
   </hyperlinks>
-  <drawing r:id="rId154"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>